<commit_message>
Refactor XML tree UI and relation label logic
Move XML_Tags_Schema.xlsx into public/docs (adds temp ~$ file). Update XmlTreeNode UI: tweak mandatory config (conditional border solid), inline node description, replace Repeat icon with a textual multiple indicator and color adjustments, remove group badge, use Info icon for conditions and expand tooltip layout. Refactor resolveRelationLabel in XmlSchema.tsx: introduce formatTag/formatGroup helpers, build source and target labels that support group IDs and attribute tags, and improve handling of missing targets. These changes improve relation labeling correctness and node display clarity.
</commit_message>
<xml_diff>
--- a/public/docs/XML_Tags_Schema.xlsx
+++ b/public/docs/XML_Tags_Schema.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\My-Python-Hub\GithubRepos\mft1998-portfolio\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\My-Python-Hub\GithubRepos\mft1998-portfolio\public\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B80DAC1-D3CF-4C27-9F9E-E9E0A5C117C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4891B058-3DB0-4588-848B-AF44CAA38D14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14400" windowHeight="15600" xr2:uid="{18F53C85-61FE-4B9A-B576-452BD9DB7FDE}"/>
+    <workbookView xWindow="6135" yWindow="2655" windowWidth="19095" windowHeight="11385" xr2:uid="{18F53C85-61FE-4B9A-B576-452BD9DB7FDE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -725,6 +725,9 @@
       <c r="B9" s="1" t="s">
         <v>26</v>
       </c>
+      <c r="C9" s="1">
+        <v>2</v>
+      </c>
       <c r="F9" s="1">
         <v>3</v>
       </c>

</xml_diff>

<commit_message>
Update XmlTreeNode border styles and badges
Adjust visual styling and simplify logic for XML tree nodes. Updated mandatoryConfig for types 2 (Optional) and 3 (Conditional) to use explicit 3px borders and different border styles/colors, removed the special-case double-border handling and simplified borderClass usage. Also removed the inline "attribute" badge to reduce UI clutter. Included updated XML_Tags_Schema.xlsx documentation file.
</commit_message>
<xml_diff>
--- a/public/docs/XML_Tags_Schema.xlsx
+++ b/public/docs/XML_Tags_Schema.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\My-Python-Hub\GithubRepos\mft1998-portfolio\public\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4891B058-3DB0-4588-848B-AF44CAA38D14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2437C26-DAA0-43DA-87B2-43EC3E45F6E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6135" yWindow="2655" windowWidth="19095" windowHeight="11385" xr2:uid="{18F53C85-61FE-4B9A-B576-452BD9DB7FDE}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="14400" windowHeight="15600" xr2:uid="{18F53C85-61FE-4B9A-B576-452BD9DB7FDE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="96">
   <si>
     <t>tag_id</t>
   </si>
@@ -101,9 +101,6 @@
     <t>identifies the sender’s 19-character identifying number</t>
   </si>
   <si>
-    <t>if FI &gt;&gt; GIIN Number</t>
-  </si>
-  <si>
     <t>Alpha-2 Standard "EG"</t>
   </si>
   <si>
@@ -125,9 +122,6 @@
     <t>unique ID of the previously sent report</t>
   </si>
   <si>
-    <t>mandatory if "FATCA2", "FATCA3" or "FATCA4"</t>
-  </si>
-  <si>
     <t>YYYY-MM-DD format. Do not enter future years</t>
   </si>
   <si>
@@ -183,19 +177,172 @@
   </si>
   <si>
     <t>OR</t>
+  </si>
+  <si>
+    <t>ResCountryCode</t>
+  </si>
+  <si>
+    <t>Tax Resident Country of FI</t>
+  </si>
+  <si>
+    <t>TIN</t>
+  </si>
+  <si>
+    <t>not mandatory if Limited FFI, Trust, or closely held sponsored FFI</t>
+  </si>
+  <si>
+    <t>if FI → GIIN Number</t>
+  </si>
+  <si>
+    <t>if FI or direct reporting NFFE → GIIN, EIN Otherwise</t>
+  </si>
+  <si>
+    <t>Tax Identification Number</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Address</t>
+  </si>
+  <si>
+    <t>FilerCategory</t>
+  </si>
+  <si>
+    <t>DocSpec</t>
+  </si>
+  <si>
+    <t>FATCA601 → 606 + 610, 611</t>
+  </si>
+  <si>
+    <t>CountryCode</t>
+  </si>
+  <si>
+    <t>AddressFree</t>
+  </si>
+  <si>
+    <t>AddressFix</t>
+  </si>
+  <si>
+    <t>not allowed if Sponsored FFI, Sponsored Direct Reporting NFFE, or Trust</t>
+  </si>
+  <si>
+    <t>mandatory if no AddressFix, Both can exist</t>
+  </si>
+  <si>
+    <t>mandatory if no AddressFree, Both can exist</t>
+  </si>
+  <si>
+    <t>XOR</t>
+  </si>
+  <si>
+    <t>Pre-defined Address Format</t>
+  </si>
+  <si>
+    <t>Free Text Address</t>
+  </si>
+  <si>
+    <t>DocTypeIndic</t>
+  </si>
+  <si>
+    <t>DocRefID</t>
+  </si>
+  <si>
+    <t>mandatory if DocTypeInd is  Corr "FATCA2", Void "FATCA3" or Amnd "FATCA4"</t>
+  </si>
+  <si>
+    <t>CorrDocRefID</t>
+  </si>
+  <si>
+    <t>Document's unique ID</t>
+  </si>
+  <si>
+    <t>Document's Type</t>
+  </si>
+  <si>
+    <t>New → FATCA 1, Corr → FATCA2, Void → FATCA3 or Amnd → FATCA4</t>
+  </si>
+  <si>
+    <t>NoAccountToReport</t>
+  </si>
+  <si>
+    <t>Always "yes"</t>
+  </si>
+  <si>
+    <t>AccountNumber</t>
+  </si>
+  <si>
+    <t>AccountClosed</t>
+  </si>
+  <si>
+    <t>AccountHolder</t>
+  </si>
+  <si>
+    <t>SubstantialOwner</t>
+  </si>
+  <si>
+    <t>AccountBalance</t>
+  </si>
+  <si>
+    <t>Payment</t>
+  </si>
+  <si>
+    <t>CARRef</t>
+  </si>
+  <si>
+    <t>AdditionalData</t>
+  </si>
+  <si>
+    <t>AccNumberType</t>
+  </si>
+  <si>
+    <t>OECD601 → 605</t>
+  </si>
+  <si>
+    <t>Individual</t>
+  </si>
+  <si>
+    <t>Organization</t>
+  </si>
+  <si>
+    <t>AccountHolder Type</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>mandatory if AccountHolder is Organization</t>
+  </si>
+  <si>
+    <t>FATCA101 → 105</t>
+  </si>
+  <si>
+    <t>currCode</t>
+  </si>
+  <si>
+    <t>3-letter currency code "USD"</t>
+  </si>
+  <si>
+    <t>can be +ve, 0, -ve</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -218,9 +365,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -537,7 +690,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C42EF740-40BD-4580-AA1E-7E614CAA4224}">
-  <dimension ref="A1:M35"/>
+  <dimension ref="A1:M61"/>
   <sheetFormatPr defaultColWidth="17.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.42578125" style="1" customWidth="1"/>
@@ -584,13 +737,13 @@
         <v>7</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="30" x14ac:dyDescent="0.25">
@@ -644,7 +797,7 @@
         <v>20</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>21</v>
+        <v>51</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
@@ -661,7 +814,7 @@
         <v>1</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
@@ -678,7 +831,7 @@
         <v>1</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
@@ -695,7 +848,7 @@
         <v>1</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="60" x14ac:dyDescent="0.25">
@@ -712,18 +865,18 @@
         <v>1</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" ht="75" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C9" s="1">
         <v>2</v>
@@ -732,10 +885,10 @@
         <v>3</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>29</v>
+        <v>70</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="45" x14ac:dyDescent="0.25">
@@ -752,10 +905,10 @@
         <v>1</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="45" x14ac:dyDescent="0.25">
@@ -772,10 +925,10 @@
         <v>1</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
@@ -783,7 +936,7 @@
         <v>11</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C12" s="1">
         <v>1</v>
@@ -797,7 +950,7 @@
         <v>12</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C13" s="1">
         <v>11</v>
@@ -811,7 +964,7 @@
         <v>13</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C14" s="1">
         <v>11</v>
@@ -825,7 +978,7 @@
         <v>14</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C15" s="1">
         <v>13</v>
@@ -834,13 +987,13 @@
         <v>3</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="K15" s="1" t="s">
-        <v>48</v>
+        <v>43</v>
+      </c>
+      <c r="K15" s="2" t="s">
+        <v>65</v>
       </c>
       <c r="L15" s="1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="16" spans="1:12" ht="75" x14ac:dyDescent="0.25">
@@ -848,7 +1001,7 @@
         <v>15</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C16" s="1">
         <v>13</v>
@@ -860,16 +1013,16 @@
         <v>3</v>
       </c>
       <c r="G16" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="H16" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="H16" s="1" t="s">
-        <v>46</v>
-      </c>
       <c r="J16" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="K16" s="1" t="s">
-        <v>48</v>
+        <v>41</v>
+      </c>
+      <c r="K16" s="2" t="s">
+        <v>65</v>
       </c>
       <c r="L16" s="1">
         <v>14</v>
@@ -880,7 +1033,7 @@
         <v>16</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C17" s="1">
         <v>13</v>
@@ -892,109 +1045,713 @@
         <v>3</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="J17" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="K17" s="1" t="s">
-        <v>48</v>
+        <v>41</v>
+      </c>
+      <c r="K17" s="2" t="s">
+        <v>65</v>
       </c>
       <c r="L17" s="1">
         <v>14</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>17</v>
       </c>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B18" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C18" s="1">
+        <v>12</v>
+      </c>
+      <c r="F18" s="1">
+        <v>2</v>
+      </c>
+      <c r="H18" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="I18" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" ht="60" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
         <v>18</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C19" s="1">
+        <v>12</v>
+      </c>
+      <c r="F19" s="1">
+        <v>3</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="H19" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="I19" s="1" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <v>19</v>
       </c>
+      <c r="B20" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C20" s="1">
+        <v>12</v>
+      </c>
+      <c r="F20" s="1">
+        <v>1</v>
+      </c>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
         <v>20</v>
       </c>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B21" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C21" s="1">
+        <v>12</v>
+      </c>
+      <c r="F21" s="1">
+        <v>1</v>
+      </c>
+      <c r="I21" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" ht="75" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
         <v>21</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C22" s="1">
+        <v>12</v>
+      </c>
+      <c r="F22" s="1">
+        <v>3</v>
+      </c>
+      <c r="G22" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="I22" s="1" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
         <v>22</v>
       </c>
+      <c r="B23" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C23" s="1">
+        <v>12</v>
+      </c>
+      <c r="F23" s="1">
+        <v>1</v>
+      </c>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
         <v>23</v>
       </c>
-    </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B24" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C24" s="1">
+        <v>20</v>
+      </c>
+      <c r="F24" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
         <v>24</v>
       </c>
-    </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B25" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C25" s="1">
+        <v>20</v>
+      </c>
+      <c r="F25" s="1">
+        <v>3</v>
+      </c>
+      <c r="G25" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="H25" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="K25" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="L25" s="1">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
         <v>25</v>
       </c>
-    </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B26" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C26" s="1">
+        <v>20</v>
+      </c>
+      <c r="F26" s="1">
+        <v>3</v>
+      </c>
+      <c r="G26" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="H26" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="K26" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="L26" s="1">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" ht="60" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
         <v>26</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C27" s="1">
+        <v>22</v>
+      </c>
+      <c r="F27" s="1">
+        <v>1</v>
+      </c>
+      <c r="H27" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="I27" s="1" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
         <v>27</v>
       </c>
-    </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B28" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C28" s="1">
+        <v>22</v>
+      </c>
+      <c r="F28" s="1">
+        <v>1</v>
+      </c>
+      <c r="H28" s="1" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" ht="75" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
         <v>28</v>
       </c>
-    </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B29" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C29" s="1">
+        <v>22</v>
+      </c>
+      <c r="F29" s="1">
+        <v>3</v>
+      </c>
+      <c r="G29" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="H29" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" ht="75" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
         <v>29</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="C30" s="1">
+        <v>22</v>
+      </c>
+      <c r="F30" s="1">
+        <v>3</v>
+      </c>
+      <c r="G30" s="1" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
         <v>30</v>
       </c>
-    </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B31" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C31" s="1">
+        <v>14</v>
+      </c>
+      <c r="F31" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" ht="60" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
         <v>31</v>
       </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B32" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C32" s="1">
+        <v>30</v>
+      </c>
+      <c r="F32" s="1">
+        <v>1</v>
+      </c>
+      <c r="H32" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="I32" s="1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
         <v>32</v>
       </c>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B33" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C33" s="1">
+        <v>30</v>
+      </c>
+      <c r="F33" s="1">
+        <v>1</v>
+      </c>
+      <c r="H33" s="1" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" ht="75" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
         <v>33</v>
       </c>
-    </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B34" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C34" s="1">
+        <v>30</v>
+      </c>
+      <c r="F34" s="1">
+        <v>3</v>
+      </c>
+      <c r="G34" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="H34" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" ht="75" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
         <v>34</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="C35" s="1">
+        <v>30</v>
+      </c>
+      <c r="F35" s="1">
+        <v>3</v>
+      </c>
+      <c r="G35" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A36" s="1">
+        <v>35</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C36" s="1">
+        <v>14</v>
+      </c>
+      <c r="F36" s="1">
+        <v>1</v>
+      </c>
+      <c r="I36" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A37" s="1">
+        <v>36</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C37" s="1">
+        <v>15</v>
+      </c>
+      <c r="F37" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="A38" s="1">
+        <v>37</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C38" s="1">
+        <v>36</v>
+      </c>
+      <c r="F38" s="1">
+        <v>1</v>
+      </c>
+      <c r="H38" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="I38" s="1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A39" s="1">
+        <v>38</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C39" s="1">
+        <v>36</v>
+      </c>
+      <c r="F39" s="1">
+        <v>1</v>
+      </c>
+      <c r="H39" s="1" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+      <c r="A40" s="1">
+        <v>39</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C40" s="1">
+        <v>36</v>
+      </c>
+      <c r="F40" s="1">
+        <v>3</v>
+      </c>
+      <c r="G40" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="H40" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+      <c r="A41" s="1">
+        <v>40</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="C41" s="1">
+        <v>36</v>
+      </c>
+      <c r="F41" s="1">
+        <v>3</v>
+      </c>
+      <c r="G41" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A42" s="1">
+        <v>41</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C42" s="1">
+        <v>15</v>
+      </c>
+      <c r="F42" s="1">
+        <v>1</v>
+      </c>
+      <c r="I42" s="1" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A43" s="1">
+        <v>42</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C43" s="1">
+        <v>41</v>
+      </c>
+      <c r="D43" s="1">
+        <v>1</v>
+      </c>
+      <c r="F43" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A44" s="1">
+        <v>43</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C44" s="1">
+        <v>15</v>
+      </c>
+      <c r="F44" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A45" s="1">
+        <v>44</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C45" s="1">
+        <v>15</v>
+      </c>
+      <c r="F45" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A46" s="1">
+        <v>45</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C46" s="1">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A47" s="1">
+        <v>46</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C47" s="1">
+        <v>15</v>
+      </c>
+      <c r="F47" s="1">
+        <v>1</v>
+      </c>
+      <c r="I47" s="1" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A48" s="1">
+        <v>47</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C48" s="1">
+        <v>15</v>
+      </c>
+      <c r="E48" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A49" s="1">
+        <v>48</v>
+      </c>
+      <c r="B49" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C49" s="1">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="50" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A50" s="1">
+        <v>49</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C50" s="1">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="51" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A51" s="1">
+        <v>50</v>
+      </c>
+      <c r="B51" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C51" s="1">
+        <v>44</v>
+      </c>
+      <c r="F51" s="1">
+        <v>3</v>
+      </c>
+      <c r="K51" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="L51" s="1" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="52" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A52" s="1">
+        <v>51</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="C52" s="1">
+        <v>44</v>
+      </c>
+      <c r="F52" s="1">
+        <v>3</v>
+      </c>
+      <c r="J52" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="K52" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="L52" s="1">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="53" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="A53" s="1">
+        <v>52</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C53" s="1">
+        <v>44</v>
+      </c>
+      <c r="F53" s="1">
+        <v>3</v>
+      </c>
+      <c r="G53" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I53" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="J53" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="K53" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="L53" s="1">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="54" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A54" s="1">
+        <v>53</v>
+      </c>
+      <c r="B54" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="C54" s="1">
+        <v>46</v>
+      </c>
+      <c r="D54" s="1">
+        <v>1</v>
+      </c>
+      <c r="F54" s="1">
+        <v>1</v>
+      </c>
+      <c r="I54" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="55" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A55" s="1">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="56" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A56" s="1">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="57" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A57" s="1">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="58" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A58" s="1">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="59" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A59" s="1">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="60" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A60" s="1">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="61" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A61" s="1">
+        <v>60</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add 'Hide Attributes' filter and UI switch
Introduce a new hideAttribute state in XmlSchema, include it in the data filtering logic and effect dependency array so attribute tags can be excluded from the tree. Add a corresponding Switch and Label to the UI controls. Also update the public/docs/XML_Tags_Schema.xlsx binary (refreshed schema source).
</commit_message>
<xml_diff>
--- a/public/docs/XML_Tags_Schema.xlsx
+++ b/public/docs/XML_Tags_Schema.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\My-Python-Hub\GithubRepos\mft1998-portfolio\public\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2309ED6C-A74A-4DBF-8A1D-AB20079FD20F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13C0F2BF-B4C7-4902-ACE7-51DB45C7D4D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{18F53C85-61FE-4B9A-B576-452BD9DB7FDE}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="14400" windowHeight="15600" xr2:uid="{18F53C85-61FE-4B9A-B576-452BD9DB7FDE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -388,7 +388,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -401,6 +401,14 @@
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -423,7 +431,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -432,6 +440,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1613,7 +1624,7 @@
       <c r="D43" s="1">
         <v>1</v>
       </c>
-      <c r="F43" s="1">
+      <c r="F43" s="4">
         <v>2</v>
       </c>
     </row>
@@ -1655,6 +1666,9 @@
       <c r="C46" s="1">
         <v>15</v>
       </c>
+      <c r="F46" s="1">
+        <v>2</v>
+      </c>
     </row>
     <row r="47" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A47" s="1">
@@ -1686,6 +1700,9 @@
       <c r="E48" s="1">
         <v>1</v>
       </c>
+      <c r="F48" s="1">
+        <v>2</v>
+      </c>
       <c r="H48" s="1" t="s">
         <v>98</v>
       </c>
@@ -1700,6 +1717,9 @@
       <c r="C49" s="1">
         <v>15</v>
       </c>
+      <c r="F49" s="1">
+        <v>2</v>
+      </c>
     </row>
     <row r="50" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A50" s="1">
@@ -1711,6 +1731,9 @@
       <c r="C50" s="1">
         <v>15</v>
       </c>
+      <c r="F50" s="1">
+        <v>2</v>
+      </c>
     </row>
     <row r="51" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A51" s="1">
@@ -1814,7 +1837,7 @@
       <c r="C55" s="1">
         <v>50</v>
       </c>
-      <c r="F55" s="1">
+      <c r="F55" s="4">
         <v>2</v>
       </c>
       <c r="H55" s="1" t="s">
@@ -1860,7 +1883,7 @@
       <c r="D57" s="1">
         <v>1</v>
       </c>
-      <c r="F57" s="1">
+      <c r="F57" s="4">
         <v>2</v>
       </c>
     </row>
@@ -1905,7 +1928,7 @@
       <c r="C60" s="1">
         <v>50</v>
       </c>
-      <c r="F60" s="1">
+      <c r="F60" s="4">
         <v>2</v>
       </c>
     </row>
@@ -2117,6 +2140,9 @@
       </c>
       <c r="C72" s="1">
         <v>16</v>
+      </c>
+      <c r="F72" s="1">
+        <v>1</v>
       </c>
       <c r="H72" s="1" t="s">
         <v>109</v>

</xml_diff>